<commit_message>
Fix Windows compatibility and silent data-loss issues in usage dashboard
- Fix Mac-only strftime code that crashed the script entirely on Windows
- Add a daily load/match report (files loaded/skipped, schools dropped,
  freshness check) so a bad run is visible instead of silent
- Add fuzzy school-name matching as a safety net for spelling drift,
  with a conservative threshold/margin tuned against a real false-positive
- Fix quiet-days calculation to anchor on the newest snapshot date instead
  of wall-clock now(), which was inflating "days quiet" on every school
- Add tolerant column-header matching so a header typo no longer silently
  drops an entire day's file
- Correct the 13-04-2026 snapshot export (recovers 37 previously-dropped
  login rows) and add the missing 17-08-2026 snapshot
- Add run_usage_dashboard.bat as a one-click Windows runner
</commit_message>
<xml_diff>
--- a/daily_snapshots/Daily Usage Snapshot - 13-04-2026.xlsx
+++ b/daily_snapshots/Daily Usage Snapshot - 13-04-2026.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\BrandonBobbs\Desktop\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{D7EA1AD1-DF99-4FAC-9E75-C1B5FBFE612D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{18BCFE4D-CA10-4736-BA0B-1FB27302CA45}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="780" yWindow="780" windowWidth="21600" windowHeight="11295" activeTab="1" xr2:uid="{7093DCCB-0AA6-46FA-9677-4B2493DAE749}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{7093DCCB-0AA6-46FA-9677-4B2493DAE749}"/>
   </bookViews>
   <sheets>
     <sheet name="Raw Data" sheetId="1" r:id="rId1"/>
@@ -21,7 +21,7 @@
   </definedNames>
   <calcPr calcId="191029"/>
   <pivotCaches>
-    <pivotCache cacheId="7" r:id="rId3"/>
+    <pivotCache cacheId="0" r:id="rId3"/>
   </pivotCaches>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -639,9 +639,6 @@
     <t>Monday, 13 April 2026 at 06:55</t>
   </si>
   <si>
-    <t>Emai Address</t>
-  </si>
-  <si>
     <t>First Name</t>
   </si>
   <si>
@@ -805,6 +802,9 @@
   </si>
   <si>
     <t>SoniqueTheron</t>
+  </si>
+  <si>
+    <t>Email Address</t>
   </si>
 </sst>
 </file>
@@ -863,7 +863,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
@@ -874,7 +874,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" indent="2"/>
     </xf>
@@ -1489,7 +1488,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{25092182-0559-462A-85E4-BB95382CB629}" name="PivotTable1" cacheId="7" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{25092182-0559-462A-85E4-BB95382CB629}" name="PivotTable1" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
   <location ref="A3:E76" firstHeaderRow="1" firstDataRow="2" firstDataCol="1" rowPageCount="1" colPageCount="1"/>
   <pivotFields count="10">
     <pivotField showAll="0"/>
@@ -2209,34 +2208,34 @@
   <sheetData>
     <row r="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="B1" s="1" t="s">
+        <v>253</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>198</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="D1" s="1" t="s">
         <v>199</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="E1" s="1" t="s">
+        <v>211</v>
+      </c>
+      <c r="F1" s="1" t="s">
         <v>200</v>
       </c>
-      <c r="E1" s="1" t="s">
-        <v>212</v>
-      </c>
-      <c r="F1" s="1" t="s">
+      <c r="G1" s="1" t="s">
         <v>201</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="H1" s="1" t="s">
         <v>202</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="I1" s="1" t="s">
         <v>203</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="J1" s="1" t="s">
         <v>204</v>
-      </c>
-      <c r="J1" s="1" t="s">
-        <v>205</v>
       </c>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.25">
@@ -2266,10 +2265,10 @@
         <v>6</v>
       </c>
       <c r="I2" s="2" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="J2" s="2" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.25">
@@ -2299,10 +2298,10 @@
         <v>6</v>
       </c>
       <c r="I3" s="2" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="J3" s="2" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.25">
@@ -2332,10 +2331,10 @@
         <v>17</v>
       </c>
       <c r="I4" s="2" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="J4" s="2" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.25">
@@ -2365,10 +2364,10 @@
         <v>23</v>
       </c>
       <c r="I5" s="2" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="J5" s="2" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.25">
@@ -2395,13 +2394,13 @@
         <v>28</v>
       </c>
       <c r="H6" s="2" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="I6" s="2" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="J6" s="2" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.25">
@@ -2431,10 +2430,10 @@
         <v>34</v>
       </c>
       <c r="I7" s="2" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="J7" s="2" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
     </row>
     <row r="8" spans="1:10" x14ac:dyDescent="0.25">
@@ -2464,10 +2463,10 @@
         <v>34</v>
       </c>
       <c r="I8" s="2" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="J8" s="2" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
     </row>
     <row r="9" spans="1:10" x14ac:dyDescent="0.25">
@@ -2497,10 +2496,10 @@
         <v>34</v>
       </c>
       <c r="I9" s="2" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="J9" s="2" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
     </row>
     <row r="10" spans="1:10" x14ac:dyDescent="0.25">
@@ -2530,10 +2529,10 @@
         <v>50</v>
       </c>
       <c r="I10" s="2" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="J10" s="2" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
     </row>
     <row r="11" spans="1:10" x14ac:dyDescent="0.25">
@@ -2563,10 +2562,10 @@
         <v>56</v>
       </c>
       <c r="I11" s="2" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="J11" s="2" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.25">
@@ -2596,10 +2595,10 @@
         <v>62</v>
       </c>
       <c r="I12" s="2" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="J12" s="2" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
     </row>
     <row r="13" spans="1:10" x14ac:dyDescent="0.25">
@@ -2629,10 +2628,10 @@
         <v>68</v>
       </c>
       <c r="I13" s="2" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="J13" s="2" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
     </row>
     <row r="14" spans="1:10" x14ac:dyDescent="0.25">
@@ -2662,10 +2661,10 @@
         <v>75</v>
       </c>
       <c r="I14" s="2" t="s">
+        <v>209</v>
+      </c>
+      <c r="J14" s="2" t="s">
         <v>210</v>
-      </c>
-      <c r="J14" s="2" t="s">
-        <v>211</v>
       </c>
     </row>
     <row r="15" spans="1:10" x14ac:dyDescent="0.25">
@@ -2695,10 +2694,10 @@
         <v>80</v>
       </c>
       <c r="I15" s="2" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="J15" s="2" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
     </row>
     <row r="16" spans="1:10" x14ac:dyDescent="0.25">
@@ -2728,10 +2727,10 @@
         <v>86</v>
       </c>
       <c r="I16" s="2" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="J16" s="2" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
     </row>
     <row r="17" spans="1:10" x14ac:dyDescent="0.25">
@@ -2761,10 +2760,10 @@
         <v>75</v>
       </c>
       <c r="I17" s="2" t="s">
+        <v>209</v>
+      </c>
+      <c r="J17" s="2" t="s">
         <v>210</v>
-      </c>
-      <c r="J17" s="2" t="s">
-        <v>211</v>
       </c>
     </row>
     <row r="18" spans="1:10" x14ac:dyDescent="0.25">
@@ -2794,10 +2793,10 @@
         <v>97</v>
       </c>
       <c r="I18" s="2" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="J18" s="2" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
     </row>
     <row r="19" spans="1:10" x14ac:dyDescent="0.25">
@@ -2824,13 +2823,13 @@
         <v>102</v>
       </c>
       <c r="H19" s="2" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="I19" s="2" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="J19" s="2" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
     </row>
     <row r="20" spans="1:10" x14ac:dyDescent="0.25">
@@ -2860,10 +2859,10 @@
         <v>6</v>
       </c>
       <c r="I20" s="2" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="J20" s="2" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
     </row>
     <row r="21" spans="1:10" x14ac:dyDescent="0.25">
@@ -2893,10 +2892,10 @@
         <v>113</v>
       </c>
       <c r="I21" s="2" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="J21" s="2" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
     </row>
     <row r="22" spans="1:10" x14ac:dyDescent="0.25">
@@ -2923,13 +2922,13 @@
         <v>118</v>
       </c>
       <c r="H22" s="2" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="I22" s="2" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="J22" s="2" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
     </row>
     <row r="23" spans="1:10" x14ac:dyDescent="0.25">
@@ -2959,10 +2958,10 @@
         <v>75</v>
       </c>
       <c r="I23" s="2" t="s">
+        <v>209</v>
+      </c>
+      <c r="J23" s="2" t="s">
         <v>210</v>
-      </c>
-      <c r="J23" s="2" t="s">
-        <v>211</v>
       </c>
     </row>
     <row r="24" spans="1:10" x14ac:dyDescent="0.25">
@@ -2992,10 +2991,10 @@
         <v>62</v>
       </c>
       <c r="I24" s="2" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="J24" s="2" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
     </row>
     <row r="25" spans="1:10" x14ac:dyDescent="0.25">
@@ -3022,13 +3021,13 @@
         <v>132</v>
       </c>
       <c r="H25" s="2" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="I25" s="2" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="J25" s="2" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
     </row>
     <row r="26" spans="1:10" x14ac:dyDescent="0.25">
@@ -3055,13 +3054,13 @@
         <v>134</v>
       </c>
       <c r="H26" s="2" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="I26" s="2" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="J26" s="2" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
     </row>
     <row r="27" spans="1:10" x14ac:dyDescent="0.25">
@@ -3091,10 +3090,10 @@
         <v>75</v>
       </c>
       <c r="I27" s="2" t="s">
+        <v>209</v>
+      </c>
+      <c r="J27" s="2" t="s">
         <v>210</v>
-      </c>
-      <c r="J27" s="2" t="s">
-        <v>211</v>
       </c>
     </row>
     <row r="28" spans="1:10" x14ac:dyDescent="0.25">
@@ -3124,10 +3123,10 @@
         <v>145</v>
       </c>
       <c r="I28" s="2" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="J28" s="2" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
     </row>
     <row r="29" spans="1:10" x14ac:dyDescent="0.25">
@@ -3157,10 +3156,10 @@
         <v>75</v>
       </c>
       <c r="I29" s="2" t="s">
+        <v>209</v>
+      </c>
+      <c r="J29" s="2" t="s">
         <v>210</v>
-      </c>
-      <c r="J29" s="2" t="s">
-        <v>211</v>
       </c>
     </row>
     <row r="30" spans="1:10" x14ac:dyDescent="0.25">
@@ -3190,10 +3189,10 @@
         <v>75</v>
       </c>
       <c r="I30" s="2" t="s">
+        <v>209</v>
+      </c>
+      <c r="J30" s="2" t="s">
         <v>210</v>
-      </c>
-      <c r="J30" s="2" t="s">
-        <v>211</v>
       </c>
     </row>
     <row r="31" spans="1:10" x14ac:dyDescent="0.25">
@@ -3223,10 +3222,10 @@
         <v>62</v>
       </c>
       <c r="I31" s="2" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="J31" s="2" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
     </row>
     <row r="32" spans="1:10" x14ac:dyDescent="0.25">
@@ -3256,10 +3255,10 @@
         <v>23</v>
       </c>
       <c r="I32" s="2" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="J32" s="2" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
     </row>
     <row r="33" spans="1:10" x14ac:dyDescent="0.25">
@@ -3289,10 +3288,10 @@
         <v>171</v>
       </c>
       <c r="I33" s="2" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="J33" s="2" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
     </row>
     <row r="34" spans="1:10" x14ac:dyDescent="0.25">
@@ -3319,13 +3318,13 @@
         <v>176</v>
       </c>
       <c r="H34" s="2" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="I34" s="2" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="J34" s="2" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
     </row>
     <row r="35" spans="1:10" x14ac:dyDescent="0.25">
@@ -3355,10 +3354,10 @@
         <v>75</v>
       </c>
       <c r="I35" s="2" t="s">
+        <v>209</v>
+      </c>
+      <c r="J35" s="2" t="s">
         <v>210</v>
-      </c>
-      <c r="J35" s="2" t="s">
-        <v>211</v>
       </c>
     </row>
     <row r="36" spans="1:10" x14ac:dyDescent="0.25">
@@ -3388,10 +3387,10 @@
         <v>50</v>
       </c>
       <c r="I36" s="2" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="J36" s="2" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
     </row>
     <row r="37" spans="1:10" x14ac:dyDescent="0.25">
@@ -3421,10 +3420,10 @@
         <v>192</v>
       </c>
       <c r="I37" s="2" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="J37" s="2" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
     </row>
     <row r="38" spans="1:10" x14ac:dyDescent="0.25">
@@ -3454,10 +3453,10 @@
         <v>86</v>
       </c>
       <c r="I38" s="2" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="J38" s="2" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
     </row>
   </sheetData>
@@ -3480,23 +3479,23 @@
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="B1" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="B4" t="s">
         <v>73</v>
@@ -3508,181 +3507,158 @@
         <v>4</v>
       </c>
       <c r="E4" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" s="4" t="s">
         <v>34</v>
       </c>
-      <c r="B5" s="6"/>
-      <c r="C5" s="6">
-        <v>1</v>
-      </c>
-      <c r="D5" s="6">
+      <c r="C5">
+        <v>1</v>
+      </c>
+      <c r="D5">
         <v>2</v>
       </c>
-      <c r="E5" s="6">
+      <c r="E5">
         <v>3</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" s="5" t="s">
-        <v>207</v>
-      </c>
-      <c r="B6" s="6"/>
-      <c r="C6" s="6">
-        <v>1</v>
-      </c>
-      <c r="D6" s="6">
+        <v>206</v>
+      </c>
+      <c r="C6">
+        <v>1</v>
+      </c>
+      <c r="D6">
         <v>2</v>
       </c>
-      <c r="E6" s="6">
+      <c r="E6">
         <v>3</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A7" s="7" t="s">
+      <c r="A7" s="6" t="s">
+        <v>217</v>
+      </c>
+      <c r="C7">
+        <v>1</v>
+      </c>
+      <c r="E7">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A8" s="6" t="s">
         <v>218</v>
       </c>
-      <c r="B7" s="6"/>
-      <c r="C7" s="6">
-        <v>1</v>
-      </c>
-      <c r="D7" s="6"/>
-      <c r="E7" s="6">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A8" s="7" t="s">
+      <c r="D8">
+        <v>1</v>
+      </c>
+      <c r="E8">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A9" s="6" t="s">
         <v>219</v>
       </c>
-      <c r="B8" s="6"/>
-      <c r="C8" s="6"/>
-      <c r="D8" s="6">
-        <v>1</v>
-      </c>
-      <c r="E8" s="6">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A9" s="7" t="s">
-        <v>220</v>
-      </c>
-      <c r="B9" s="6"/>
-      <c r="C9" s="6"/>
-      <c r="D9" s="6">
-        <v>1</v>
-      </c>
-      <c r="E9" s="6">
+      <c r="D9">
+        <v>1</v>
+      </c>
+      <c r="E9">
         <v>1</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A10" s="4" t="s">
-        <v>209</v>
-      </c>
-      <c r="B10" s="6">
+        <v>208</v>
+      </c>
+      <c r="B10">
         <v>5</v>
       </c>
-      <c r="C10" s="6"/>
-      <c r="D10" s="6">
-        <v>1</v>
-      </c>
-      <c r="E10" s="6">
+      <c r="D10">
+        <v>1</v>
+      </c>
+      <c r="E10">
         <v>6</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A11" s="5" t="s">
-        <v>208</v>
-      </c>
-      <c r="B11" s="6"/>
-      <c r="C11" s="6"/>
-      <c r="D11" s="6">
-        <v>1</v>
-      </c>
-      <c r="E11" s="6">
+        <v>207</v>
+      </c>
+      <c r="D11">
+        <v>1</v>
+      </c>
+      <c r="E11">
         <v>1</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A12" s="7" t="s">
-        <v>221</v>
-      </c>
-      <c r="B12" s="6"/>
-      <c r="C12" s="6"/>
-      <c r="D12" s="6">
-        <v>1</v>
-      </c>
-      <c r="E12" s="6">
+      <c r="A12" s="6" t="s">
+        <v>220</v>
+      </c>
+      <c r="D12">
+        <v>1</v>
+      </c>
+      <c r="E12">
         <v>1</v>
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A13" s="5" t="s">
-        <v>207</v>
-      </c>
-      <c r="B13" s="6">
+        <v>206</v>
+      </c>
+      <c r="B13">
         <v>5</v>
       </c>
-      <c r="C13" s="6"/>
-      <c r="D13" s="6"/>
-      <c r="E13" s="6">
+      <c r="E13">
         <v>5</v>
       </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A14" s="7" t="s">
+      <c r="A14" s="6" t="s">
+        <v>221</v>
+      </c>
+      <c r="B14">
+        <v>1</v>
+      </c>
+      <c r="E14">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A15" s="6" t="s">
         <v>222</v>
       </c>
-      <c r="B14" s="6">
-        <v>1</v>
-      </c>
-      <c r="C14" s="6"/>
-      <c r="D14" s="6"/>
-      <c r="E14" s="6">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A15" s="7" t="s">
+      <c r="B15">
+        <v>2</v>
+      </c>
+      <c r="E15">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A16" s="6" t="s">
         <v>223</v>
       </c>
-      <c r="B15" s="6">
-        <v>2</v>
-      </c>
-      <c r="C15" s="6"/>
-      <c r="D15" s="6"/>
-      <c r="E15" s="6">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A16" s="7" t="s">
+      <c r="B16">
+        <v>1</v>
+      </c>
+      <c r="E16">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A17" s="6" t="s">
         <v>224</v>
       </c>
-      <c r="B16" s="6">
-        <v>1</v>
-      </c>
-      <c r="C16" s="6"/>
-      <c r="D16" s="6"/>
-      <c r="E16" s="6">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A17" s="7" t="s">
-        <v>225</v>
-      </c>
-      <c r="B17" s="6">
-        <v>1</v>
-      </c>
-      <c r="C17" s="6"/>
-      <c r="D17" s="6"/>
-      <c r="E17" s="6">
+      <c r="B17">
+        <v>1</v>
+      </c>
+      <c r="E17">
         <v>1</v>
       </c>
     </row>
@@ -3690,38 +3666,32 @@
       <c r="A18" s="4" t="s">
         <v>113</v>
       </c>
-      <c r="B18" s="6"/>
-      <c r="C18" s="6"/>
-      <c r="D18" s="6">
-        <v>1</v>
-      </c>
-      <c r="E18" s="6">
+      <c r="D18">
+        <v>1</v>
+      </c>
+      <c r="E18">
         <v>1</v>
       </c>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A19" s="5" t="s">
-        <v>207</v>
-      </c>
-      <c r="B19" s="6"/>
-      <c r="C19" s="6"/>
-      <c r="D19" s="6">
-        <v>1</v>
-      </c>
-      <c r="E19" s="6">
+        <v>206</v>
+      </c>
+      <c r="D19">
+        <v>1</v>
+      </c>
+      <c r="E19">
         <v>1</v>
       </c>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A20" s="7" t="s">
-        <v>226</v>
-      </c>
-      <c r="B20" s="6"/>
-      <c r="C20" s="6"/>
-      <c r="D20" s="6">
-        <v>1</v>
-      </c>
-      <c r="E20" s="6">
+      <c r="A20" s="6" t="s">
+        <v>225</v>
+      </c>
+      <c r="D20">
+        <v>1</v>
+      </c>
+      <c r="E20">
         <v>1</v>
       </c>
     </row>
@@ -3729,38 +3699,32 @@
       <c r="A21" s="4" t="s">
         <v>171</v>
       </c>
-      <c r="B21" s="6"/>
-      <c r="C21" s="6">
-        <v>1</v>
-      </c>
-      <c r="D21" s="6"/>
-      <c r="E21" s="6">
+      <c r="C21">
+        <v>1</v>
+      </c>
+      <c r="E21">
         <v>1</v>
       </c>
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A22" s="5" t="s">
-        <v>208</v>
-      </c>
-      <c r="B22" s="6"/>
-      <c r="C22" s="6">
-        <v>1</v>
-      </c>
-      <c r="D22" s="6"/>
-      <c r="E22" s="6">
+        <v>207</v>
+      </c>
+      <c r="C22">
+        <v>1</v>
+      </c>
+      <c r="E22">
         <v>1</v>
       </c>
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A23" s="7" t="s">
-        <v>227</v>
-      </c>
-      <c r="B23" s="6"/>
-      <c r="C23" s="6">
-        <v>1</v>
-      </c>
-      <c r="D23" s="6"/>
-      <c r="E23" s="6">
+      <c r="A23" s="6" t="s">
+        <v>226</v>
+      </c>
+      <c r="C23">
+        <v>1</v>
+      </c>
+      <c r="E23">
         <v>1</v>
       </c>
     </row>
@@ -3768,38 +3732,32 @@
       <c r="A24" s="4" t="s">
         <v>145</v>
       </c>
-      <c r="B24" s="6"/>
-      <c r="C24" s="6">
-        <v>1</v>
-      </c>
-      <c r="D24" s="6"/>
-      <c r="E24" s="6">
+      <c r="C24">
+        <v>1</v>
+      </c>
+      <c r="E24">
         <v>1</v>
       </c>
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A25" s="5" t="s">
-        <v>208</v>
-      </c>
-      <c r="B25" s="6"/>
-      <c r="C25" s="6">
-        <v>1</v>
-      </c>
-      <c r="D25" s="6"/>
-      <c r="E25" s="6">
+        <v>207</v>
+      </c>
+      <c r="C25">
+        <v>1</v>
+      </c>
+      <c r="E25">
         <v>1</v>
       </c>
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A26" s="7" t="s">
-        <v>228</v>
-      </c>
-      <c r="B26" s="6"/>
-      <c r="C26" s="6">
-        <v>1</v>
-      </c>
-      <c r="D26" s="6"/>
-      <c r="E26" s="6">
+      <c r="A26" s="6" t="s">
+        <v>227</v>
+      </c>
+      <c r="C26">
+        <v>1</v>
+      </c>
+      <c r="E26">
         <v>1</v>
       </c>
     </row>
@@ -3807,38 +3765,32 @@
       <c r="A27" s="4" t="s">
         <v>80</v>
       </c>
-      <c r="B27" s="6"/>
-      <c r="C27" s="6">
-        <v>1</v>
-      </c>
-      <c r="D27" s="6"/>
-      <c r="E27" s="6">
+      <c r="C27">
+        <v>1</v>
+      </c>
+      <c r="E27">
         <v>1</v>
       </c>
     </row>
     <row r="28" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A28" s="5" t="s">
-        <v>208</v>
-      </c>
-      <c r="B28" s="6"/>
-      <c r="C28" s="6">
-        <v>1</v>
-      </c>
-      <c r="D28" s="6"/>
-      <c r="E28" s="6">
+        <v>207</v>
+      </c>
+      <c r="C28">
+        <v>1</v>
+      </c>
+      <c r="E28">
         <v>1</v>
       </c>
     </row>
     <row r="29" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A29" s="7" t="s">
-        <v>229</v>
-      </c>
-      <c r="B29" s="6"/>
-      <c r="C29" s="6">
-        <v>1</v>
-      </c>
-      <c r="D29" s="6"/>
-      <c r="E29" s="6">
+      <c r="A29" s="6" t="s">
+        <v>228</v>
+      </c>
+      <c r="C29">
+        <v>1</v>
+      </c>
+      <c r="E29">
         <v>1</v>
       </c>
     </row>
@@ -3846,55 +3798,49 @@
       <c r="A30" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="B30" s="6"/>
-      <c r="C30" s="6">
-        <v>1</v>
-      </c>
-      <c r="D30" s="6">
-        <v>1</v>
-      </c>
-      <c r="E30" s="6">
+      <c r="C30">
+        <v>1</v>
+      </c>
+      <c r="D30">
+        <v>1</v>
+      </c>
+      <c r="E30">
         <v>2</v>
       </c>
     </row>
     <row r="31" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A31" s="5" t="s">
-        <v>208</v>
-      </c>
-      <c r="B31" s="6"/>
-      <c r="C31" s="6">
-        <v>1</v>
-      </c>
-      <c r="D31" s="6">
-        <v>1</v>
-      </c>
-      <c r="E31" s="6">
+        <v>207</v>
+      </c>
+      <c r="C31">
+        <v>1</v>
+      </c>
+      <c r="D31">
+        <v>1</v>
+      </c>
+      <c r="E31">
         <v>2</v>
       </c>
     </row>
     <row r="32" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A32" s="7" t="s">
+      <c r="A32" s="6" t="s">
+        <v>229</v>
+      </c>
+      <c r="D32">
+        <v>1</v>
+      </c>
+      <c r="E32">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="33" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A33" s="6" t="s">
         <v>230</v>
       </c>
-      <c r="B32" s="6"/>
-      <c r="C32" s="6"/>
-      <c r="D32" s="6">
-        <v>1</v>
-      </c>
-      <c r="E32" s="6">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="33" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A33" s="7" t="s">
-        <v>231</v>
-      </c>
-      <c r="B33" s="6"/>
-      <c r="C33" s="6">
-        <v>1</v>
-      </c>
-      <c r="D33" s="6"/>
-      <c r="E33" s="6">
+      <c r="C33">
+        <v>1</v>
+      </c>
+      <c r="E33">
         <v>1</v>
       </c>
     </row>
@@ -3902,38 +3848,32 @@
       <c r="A34" s="4" t="s">
         <v>68</v>
       </c>
-      <c r="B34" s="6"/>
-      <c r="C34" s="6"/>
-      <c r="D34" s="6">
-        <v>1</v>
-      </c>
-      <c r="E34" s="6">
+      <c r="D34">
+        <v>1</v>
+      </c>
+      <c r="E34">
         <v>1</v>
       </c>
     </row>
     <row r="35" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A35" s="5" t="s">
-        <v>207</v>
-      </c>
-      <c r="B35" s="6"/>
-      <c r="C35" s="6"/>
-      <c r="D35" s="6">
-        <v>1</v>
-      </c>
-      <c r="E35" s="6">
+        <v>206</v>
+      </c>
+      <c r="D35">
+        <v>1</v>
+      </c>
+      <c r="E35">
         <v>1</v>
       </c>
     </row>
     <row r="36" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A36" s="7" t="s">
-        <v>232</v>
-      </c>
-      <c r="B36" s="6"/>
-      <c r="C36" s="6"/>
-      <c r="D36" s="6">
-        <v>1</v>
-      </c>
-      <c r="E36" s="6">
+      <c r="A36" s="6" t="s">
+        <v>231</v>
+      </c>
+      <c r="D36">
+        <v>1</v>
+      </c>
+      <c r="E36">
         <v>1</v>
       </c>
     </row>
@@ -3941,38 +3881,32 @@
       <c r="A37" s="4" t="s">
         <v>97</v>
       </c>
-      <c r="B37" s="6"/>
-      <c r="C37" s="6">
-        <v>1</v>
-      </c>
-      <c r="D37" s="6"/>
-      <c r="E37" s="6">
+      <c r="C37">
+        <v>1</v>
+      </c>
+      <c r="E37">
         <v>1</v>
       </c>
     </row>
     <row r="38" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A38" s="5" t="s">
-        <v>208</v>
-      </c>
-      <c r="B38" s="6"/>
-      <c r="C38" s="6">
-        <v>1</v>
-      </c>
-      <c r="D38" s="6"/>
-      <c r="E38" s="6">
+        <v>207</v>
+      </c>
+      <c r="C38">
+        <v>1</v>
+      </c>
+      <c r="E38">
         <v>1</v>
       </c>
     </row>
     <row r="39" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A39" s="7" t="s">
-        <v>233</v>
-      </c>
-      <c r="B39" s="6"/>
-      <c r="C39" s="6">
-        <v>1</v>
-      </c>
-      <c r="D39" s="6"/>
-      <c r="E39" s="6">
+      <c r="A39" s="6" t="s">
+        <v>232</v>
+      </c>
+      <c r="C39">
+        <v>1</v>
+      </c>
+      <c r="E39">
         <v>1</v>
       </c>
     </row>
@@ -3980,68 +3914,60 @@
       <c r="A40" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="B40" s="6"/>
-      <c r="C40" s="6">
-        <v>1</v>
-      </c>
-      <c r="D40" s="6">
+      <c r="C40">
+        <v>1</v>
+      </c>
+      <c r="D40">
         <v>2</v>
       </c>
-      <c r="E40" s="6">
+      <c r="E40">
         <v>3</v>
       </c>
     </row>
     <row r="41" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A41" s="5" t="s">
-        <v>207</v>
-      </c>
-      <c r="B41" s="6"/>
-      <c r="C41" s="6">
-        <v>1</v>
-      </c>
-      <c r="D41" s="6">
+        <v>206</v>
+      </c>
+      <c r="C41">
+        <v>1</v>
+      </c>
+      <c r="D41">
         <v>2</v>
       </c>
-      <c r="E41" s="6">
+      <c r="E41">
         <v>3</v>
       </c>
     </row>
     <row r="42" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A42" s="7" t="s">
+      <c r="A42" s="6" t="s">
+        <v>233</v>
+      </c>
+      <c r="C42">
+        <v>1</v>
+      </c>
+      <c r="E42">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="43" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A43" s="6" t="s">
         <v>234</v>
       </c>
-      <c r="B42" s="6"/>
-      <c r="C42" s="6">
-        <v>1</v>
-      </c>
-      <c r="D42" s="6"/>
-      <c r="E42" s="6">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="43" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A43" s="7" t="s">
+      <c r="D43">
+        <v>1</v>
+      </c>
+      <c r="E43">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="44" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A44" s="6" t="s">
         <v>235</v>
       </c>
-      <c r="B43" s="6"/>
-      <c r="C43" s="6"/>
-      <c r="D43" s="6">
-        <v>1</v>
-      </c>
-      <c r="E43" s="6">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="44" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A44" s="7" t="s">
-        <v>236</v>
-      </c>
-      <c r="B44" s="6"/>
-      <c r="C44" s="6"/>
-      <c r="D44" s="6">
-        <v>1</v>
-      </c>
-      <c r="E44" s="6">
+      <c r="D44">
+        <v>1</v>
+      </c>
+      <c r="E44">
         <v>1</v>
       </c>
     </row>
@@ -4049,38 +3975,32 @@
       <c r="A45" s="4" t="s">
         <v>192</v>
       </c>
-      <c r="B45" s="6"/>
-      <c r="C45" s="6"/>
-      <c r="D45" s="6">
-        <v>1</v>
-      </c>
-      <c r="E45" s="6">
+      <c r="D45">
+        <v>1</v>
+      </c>
+      <c r="E45">
         <v>1</v>
       </c>
     </row>
     <row r="46" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A46" s="5" t="s">
-        <v>208</v>
-      </c>
-      <c r="B46" s="6"/>
-      <c r="C46" s="6"/>
-      <c r="D46" s="6">
-        <v>1</v>
-      </c>
-      <c r="E46" s="6">
+        <v>207</v>
+      </c>
+      <c r="D46">
+        <v>1</v>
+      </c>
+      <c r="E46">
         <v>1</v>
       </c>
     </row>
     <row r="47" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A47" s="7" t="s">
-        <v>237</v>
-      </c>
-      <c r="B47" s="6"/>
-      <c r="C47" s="6"/>
-      <c r="D47" s="6">
-        <v>1</v>
-      </c>
-      <c r="E47" s="6">
+      <c r="A47" s="6" t="s">
+        <v>236</v>
+      </c>
+      <c r="D47">
+        <v>1</v>
+      </c>
+      <c r="E47">
         <v>1</v>
       </c>
     </row>
@@ -4088,116 +4008,98 @@
       <c r="A48" s="4" t="s">
         <v>75</v>
       </c>
-      <c r="B48" s="6">
+      <c r="B48">
         <v>7</v>
       </c>
-      <c r="C48" s="6"/>
-      <c r="D48" s="6"/>
-      <c r="E48" s="6">
+      <c r="E48">
         <v>7</v>
       </c>
     </row>
     <row r="49" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A49" s="5" t="s">
-        <v>210</v>
-      </c>
-      <c r="B49" s="6">
+        <v>209</v>
+      </c>
+      <c r="B49">
         <v>7</v>
       </c>
-      <c r="C49" s="6"/>
-      <c r="D49" s="6"/>
-      <c r="E49" s="6">
+      <c r="E49">
         <v>7</v>
       </c>
     </row>
     <row r="50" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A50" s="7" t="s">
+      <c r="A50" s="6" t="s">
+        <v>237</v>
+      </c>
+      <c r="B50">
+        <v>1</v>
+      </c>
+      <c r="E50">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="51" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A51" s="6" t="s">
         <v>238</v>
       </c>
-      <c r="B50" s="6">
-        <v>1</v>
-      </c>
-      <c r="C50" s="6"/>
-      <c r="D50" s="6"/>
-      <c r="E50" s="6">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="51" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A51" s="7" t="s">
+      <c r="B51">
+        <v>1</v>
+      </c>
+      <c r="E51">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="52" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A52" s="6" t="s">
         <v>239</v>
       </c>
-      <c r="B51" s="6">
-        <v>1</v>
-      </c>
-      <c r="C51" s="6"/>
-      <c r="D51" s="6"/>
-      <c r="E51" s="6">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="52" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A52" s="7" t="s">
+      <c r="B52">
+        <v>1</v>
+      </c>
+      <c r="E52">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="53" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A53" s="6" t="s">
         <v>240</v>
       </c>
-      <c r="B52" s="6">
-        <v>1</v>
-      </c>
-      <c r="C52" s="6"/>
-      <c r="D52" s="6"/>
-      <c r="E52" s="6">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="53" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A53" s="7" t="s">
+      <c r="B53">
+        <v>1</v>
+      </c>
+      <c r="E53">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="54" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A54" s="6" t="s">
         <v>241</v>
       </c>
-      <c r="B53" s="6">
-        <v>1</v>
-      </c>
-      <c r="C53" s="6"/>
-      <c r="D53" s="6"/>
-      <c r="E53" s="6">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="54" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A54" s="7" t="s">
+      <c r="B54">
+        <v>1</v>
+      </c>
+      <c r="E54">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="55" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A55" s="6" t="s">
         <v>242</v>
       </c>
-      <c r="B54" s="6">
-        <v>1</v>
-      </c>
-      <c r="C54" s="6"/>
-      <c r="D54" s="6"/>
-      <c r="E54" s="6">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="55" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A55" s="7" t="s">
+      <c r="B55">
+        <v>1</v>
+      </c>
+      <c r="E55">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="56" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A56" s="6" t="s">
         <v>243</v>
       </c>
-      <c r="B55" s="6">
-        <v>1</v>
-      </c>
-      <c r="C55" s="6"/>
-      <c r="D55" s="6"/>
-      <c r="E55" s="6">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="56" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A56" s="7" t="s">
-        <v>244</v>
-      </c>
-      <c r="B56" s="6">
-        <v>1</v>
-      </c>
-      <c r="C56" s="6"/>
-      <c r="D56" s="6"/>
-      <c r="E56" s="6">
+      <c r="B56">
+        <v>1</v>
+      </c>
+      <c r="E56">
         <v>1</v>
       </c>
     </row>
@@ -4205,38 +4107,32 @@
       <c r="A57" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="B57" s="6"/>
-      <c r="C57" s="6">
-        <v>1</v>
-      </c>
-      <c r="D57" s="6"/>
-      <c r="E57" s="6">
+      <c r="C57">
+        <v>1</v>
+      </c>
+      <c r="E57">
         <v>1</v>
       </c>
     </row>
     <row r="58" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A58" s="5" t="s">
-        <v>208</v>
-      </c>
-      <c r="B58" s="6"/>
-      <c r="C58" s="6">
-        <v>1</v>
-      </c>
-      <c r="D58" s="6"/>
-      <c r="E58" s="6">
+        <v>207</v>
+      </c>
+      <c r="C58">
+        <v>1</v>
+      </c>
+      <c r="E58">
         <v>1</v>
       </c>
     </row>
     <row r="59" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A59" s="7" t="s">
-        <v>245</v>
-      </c>
-      <c r="B59" s="6"/>
-      <c r="C59" s="6">
-        <v>1</v>
-      </c>
-      <c r="D59" s="6"/>
-      <c r="E59" s="6">
+      <c r="A59" s="6" t="s">
+        <v>244</v>
+      </c>
+      <c r="C59">
+        <v>1</v>
+      </c>
+      <c r="E59">
         <v>1</v>
       </c>
     </row>
@@ -4244,51 +4140,43 @@
       <c r="A60" s="4" t="s">
         <v>86</v>
       </c>
-      <c r="B60" s="6"/>
-      <c r="C60" s="6"/>
-      <c r="D60" s="6">
+      <c r="D60">
         <v>2</v>
       </c>
-      <c r="E60" s="6">
+      <c r="E60">
         <v>2</v>
       </c>
     </row>
     <row r="61" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A61" s="5" t="s">
-        <v>207</v>
-      </c>
-      <c r="B61" s="6"/>
-      <c r="C61" s="6"/>
-      <c r="D61" s="6">
+        <v>206</v>
+      </c>
+      <c r="D61">
         <v>2</v>
       </c>
-      <c r="E61" s="6">
+      <c r="E61">
         <v>2</v>
       </c>
     </row>
     <row r="62" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A62" s="7" t="s">
+      <c r="A62" s="6" t="s">
+        <v>245</v>
+      </c>
+      <c r="D62">
+        <v>1</v>
+      </c>
+      <c r="E62">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="63" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A63" s="6" t="s">
         <v>246</v>
       </c>
-      <c r="B62" s="6"/>
-      <c r="C62" s="6"/>
-      <c r="D62" s="6">
-        <v>1</v>
-      </c>
-      <c r="E62" s="6">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="63" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A63" s="7" t="s">
-        <v>247</v>
-      </c>
-      <c r="B63" s="6"/>
-      <c r="C63" s="6"/>
-      <c r="D63" s="6">
-        <v>1</v>
-      </c>
-      <c r="E63" s="6">
+      <c r="D63">
+        <v>1</v>
+      </c>
+      <c r="E63">
         <v>1</v>
       </c>
     </row>
@@ -4296,38 +4184,32 @@
       <c r="A64" s="4" t="s">
         <v>56</v>
       </c>
-      <c r="B64" s="6"/>
-      <c r="C64" s="6">
-        <v>1</v>
-      </c>
-      <c r="D64" s="6"/>
-      <c r="E64" s="6">
+      <c r="C64">
+        <v>1</v>
+      </c>
+      <c r="E64">
         <v>1</v>
       </c>
     </row>
     <row r="65" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A65" s="5" t="s">
-        <v>208</v>
-      </c>
-      <c r="B65" s="6"/>
-      <c r="C65" s="6">
-        <v>1</v>
-      </c>
-      <c r="D65" s="6"/>
-      <c r="E65" s="6">
+        <v>207</v>
+      </c>
+      <c r="C65">
+        <v>1</v>
+      </c>
+      <c r="E65">
         <v>1</v>
       </c>
     </row>
     <row r="66" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A66" s="7" t="s">
-        <v>248</v>
-      </c>
-      <c r="B66" s="6"/>
-      <c r="C66" s="6">
-        <v>1</v>
-      </c>
-      <c r="D66" s="6"/>
-      <c r="E66" s="6">
+      <c r="A66" s="6" t="s">
+        <v>247</v>
+      </c>
+      <c r="C66">
+        <v>1</v>
+      </c>
+      <c r="E66">
         <v>1</v>
       </c>
     </row>
@@ -4335,51 +4217,43 @@
       <c r="A67" s="4" t="s">
         <v>50</v>
       </c>
-      <c r="B67" s="6"/>
-      <c r="C67" s="6"/>
-      <c r="D67" s="6">
+      <c r="D67">
         <v>2</v>
       </c>
-      <c r="E67" s="6">
+      <c r="E67">
         <v>2</v>
       </c>
     </row>
     <row r="68" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A68" s="5" t="s">
-        <v>207</v>
-      </c>
-      <c r="B68" s="6"/>
-      <c r="C68" s="6"/>
-      <c r="D68" s="6">
+        <v>206</v>
+      </c>
+      <c r="D68">
         <v>2</v>
       </c>
-      <c r="E68" s="6">
+      <c r="E68">
         <v>2</v>
       </c>
     </row>
     <row r="69" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A69" s="7" t="s">
+      <c r="A69" s="6" t="s">
+        <v>248</v>
+      </c>
+      <c r="D69">
+        <v>1</v>
+      </c>
+      <c r="E69">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="70" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A70" s="6" t="s">
         <v>249</v>
       </c>
-      <c r="B69" s="6"/>
-      <c r="C69" s="6"/>
-      <c r="D69" s="6">
-        <v>1</v>
-      </c>
-      <c r="E69" s="6">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="70" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A70" s="7" t="s">
-        <v>250</v>
-      </c>
-      <c r="B70" s="6"/>
-      <c r="C70" s="6"/>
-      <c r="D70" s="6">
-        <v>1</v>
-      </c>
-      <c r="E70" s="6">
+      <c r="D70">
+        <v>1</v>
+      </c>
+      <c r="E70">
         <v>1</v>
       </c>
     </row>
@@ -4387,81 +4261,71 @@
       <c r="A71" s="4" t="s">
         <v>62</v>
       </c>
-      <c r="B71" s="6"/>
-      <c r="C71" s="6"/>
-      <c r="D71" s="6">
+      <c r="D71">
         <v>3</v>
       </c>
-      <c r="E71" s="6">
+      <c r="E71">
         <v>3</v>
       </c>
     </row>
     <row r="72" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A72" s="5" t="s">
-        <v>207</v>
-      </c>
-      <c r="B72" s="6"/>
-      <c r="C72" s="6"/>
-      <c r="D72" s="6">
+        <v>206</v>
+      </c>
+      <c r="D72">
         <v>3</v>
       </c>
-      <c r="E72" s="6">
+      <c r="E72">
         <v>3</v>
       </c>
     </row>
     <row r="73" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A73" s="7" t="s">
+      <c r="A73" s="6" t="s">
+        <v>250</v>
+      </c>
+      <c r="D73">
+        <v>1</v>
+      </c>
+      <c r="E73">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="74" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A74" s="6" t="s">
         <v>251</v>
       </c>
-      <c r="B73" s="6"/>
-      <c r="C73" s="6"/>
-      <c r="D73" s="6">
-        <v>1</v>
-      </c>
-      <c r="E73" s="6">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="74" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A74" s="7" t="s">
+      <c r="D74">
+        <v>1</v>
+      </c>
+      <c r="E74">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="75" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A75" s="6" t="s">
         <v>252</v>
       </c>
-      <c r="B74" s="6"/>
-      <c r="C74" s="6"/>
-      <c r="D74" s="6">
-        <v>1</v>
-      </c>
-      <c r="E74" s="6">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="75" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A75" s="7" t="s">
-        <v>253</v>
-      </c>
-      <c r="B75" s="6"/>
-      <c r="C75" s="6"/>
-      <c r="D75" s="6">
-        <v>1</v>
-      </c>
-      <c r="E75" s="6">
+      <c r="D75">
+        <v>1</v>
+      </c>
+      <c r="E75">
         <v>1</v>
       </c>
     </row>
     <row r="76" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A76" s="4" t="s">
-        <v>214</v>
-      </c>
-      <c r="B76" s="6">
+        <v>213</v>
+      </c>
+      <c r="B76">
         <v>12</v>
       </c>
-      <c r="C76" s="6">
+      <c r="C76">
         <v>9</v>
       </c>
-      <c r="D76" s="6">
+      <c r="D76">
         <v>16</v>
       </c>
-      <c r="E76" s="6">
+      <c r="E76">
         <v>37</v>
       </c>
     </row>

</xml_diff>